<commit_message>
Add detailed consumables breakdown with unit costs per equipment (CONSUMIBLES DETALLE sheet)
https://claude.ai/code/session_019HXrhFWzWmBAKHNaDfmdYV
</commit_message>
<xml_diff>
--- a/Plan_Operaciones_M4.xlsx
+++ b/Plan_Operaciones_M4.xlsx
@@ -8,9 +8,10 @@
   </bookViews>
   <sheets>
     <sheet name="PREMISAS" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="DETALLE M4" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="RESUMEN IE" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="RESUMEN ESPECIALIDAD" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="CONSUMIBLES DETALLE" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="DETALLE M4" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="RESUMEN IE" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="RESUMEN ESPECIALIDAD" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,7 +23,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="S/. #,##0.00"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -64,8 +65,28 @@
       <color rgb="00000000"/>
       <sz val="9"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FF043941"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FF043941"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -107,8 +128,33 @@
         <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF043941"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0A7F8F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF02D47E"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -130,11 +176,25 @@
         <color rgb="00CCCCCC"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD0D0D0"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD0D0D0"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD0D0D0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD0D0D0"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -201,6 +261,63 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="10" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="8" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1159,8 +1276,9 @@
           <t>Cocina y Repostería</t>
         </is>
       </c>
-      <c r="C44" s="5" t="n">
-        <v>800</v>
+      <c r="C44" s="5">
+        <f>'CONSUMIBLES DETALLE'!F17</f>
+        <v/>
       </c>
     </row>
     <row r="45">
@@ -1169,8 +1287,9 @@
           <t>Computación e Informática</t>
         </is>
       </c>
-      <c r="C45" s="5" t="n">
-        <v>200</v>
+      <c r="C45" s="5">
+        <f>'CONSUMIBLES DETALLE'!F29</f>
+        <v/>
       </c>
     </row>
     <row r="46">
@@ -1179,8 +1298,9 @@
           <t>Construcciones Metálicas</t>
         </is>
       </c>
-      <c r="C46" s="5" t="n">
-        <v>900</v>
+      <c r="C46" s="5">
+        <f>'CONSUMIBLES DETALLE'!F45</f>
+        <v/>
       </c>
     </row>
     <row r="47">
@@ -1189,8 +1309,9 @@
           <t>Ebanistería</t>
         </is>
       </c>
-      <c r="C47" s="5" t="n">
-        <v>700</v>
+      <c r="C47" s="5">
+        <f>'CONSUMIBLES DETALLE'!F62</f>
+        <v/>
       </c>
     </row>
     <row r="48">
@@ -1199,8 +1320,9 @@
           <t>Electricidad</t>
         </is>
       </c>
-      <c r="C48" s="5" t="n">
-        <v>500</v>
+      <c r="C48" s="5">
+        <f>'CONSUMIBLES DETALLE'!F77</f>
+        <v/>
       </c>
     </row>
     <row r="49">
@@ -1209,8 +1331,9 @@
           <t>Electrónica</t>
         </is>
       </c>
-      <c r="C49" s="5" t="n">
-        <v>600</v>
+      <c r="C49" s="5">
+        <f>'CONSUMIBLES DETALLE'!F93</f>
+        <v/>
       </c>
     </row>
     <row r="50">
@@ -1219,8 +1342,9 @@
           <t>Industria Alimentaria</t>
         </is>
       </c>
-      <c r="C50" s="5" t="n">
-        <v>500</v>
+      <c r="C50" s="5">
+        <f>'CONSUMIBLES DETALLE'!F108</f>
+        <v/>
       </c>
     </row>
     <row r="51">
@@ -1229,8 +1353,9 @@
           <t>Industria del Vestido</t>
         </is>
       </c>
-      <c r="C51" s="5" t="n">
-        <v>350</v>
+      <c r="C51" s="5">
+        <f>'CONSUMIBLES DETALLE'!F123</f>
+        <v/>
       </c>
     </row>
     <row r="52">
@@ -1239,8 +1364,9 @@
           <t>Mecánica Automotriz</t>
         </is>
       </c>
-      <c r="C52" s="5" t="n">
-        <v>800</v>
+      <c r="C52" s="5">
+        <f>'CONSUMIBLES DETALLE'!F138</f>
+        <v/>
       </c>
     </row>
     <row r="54">
@@ -1297,6 +1423,3478 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F151"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>CONSUMIBLES DETALLE — COSTO UNITARIO POR EQUIPO Y ESPECIALIDAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="25" t="inlineStr">
+        <is>
+          <t>COCINA Y REPOSTERÍA</t>
+        </is>
+      </c>
+      <c r="B2" s="25" t="n"/>
+      <c r="C2" s="25" t="n"/>
+      <c r="D2" s="25" t="n"/>
+      <c r="E2" s="25" t="n"/>
+      <c r="F2" s="25" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="26" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+      <c r="B3" s="26" t="inlineStr">
+        <is>
+          <t>Consumible</t>
+        </is>
+      </c>
+      <c r="C3" s="26" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="D3" s="26" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="E3" s="26" t="inlineStr">
+        <is>
+          <t>Precio Unit. (S/.)</t>
+        </is>
+      </c>
+      <c r="F3" s="26" t="inlineStr">
+        <is>
+          <t>Subtotal</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="27" t="inlineStr">
+        <is>
+          <t>Horno convector</t>
+        </is>
+      </c>
+      <c r="B4" s="27" t="inlineStr">
+        <is>
+          <t>Gas GLP (uso operativo)</t>
+        </is>
+      </c>
+      <c r="C4" s="28" t="inlineStr">
+        <is>
+          <t>balón 10kg</t>
+        </is>
+      </c>
+      <c r="D4" s="29" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E4" s="30" t="n">
+        <v>42</v>
+      </c>
+      <c r="F4" s="30">
+        <f>D4*E4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="31" t="inlineStr">
+        <is>
+          <t>Batidora industrial</t>
+        </is>
+      </c>
+      <c r="B5" s="31" t="inlineStr">
+        <is>
+          <t>Harina sin preparar</t>
+        </is>
+      </c>
+      <c r="C5" s="32" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D5" s="33" t="n">
+        <v>8</v>
+      </c>
+      <c r="E5" s="34" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="F5" s="34">
+        <f>D5*E5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="27" t="inlineStr">
+        <is>
+          <t>Batidora industrial</t>
+        </is>
+      </c>
+      <c r="B6" s="27" t="inlineStr">
+        <is>
+          <t>Azúcar blanca</t>
+        </is>
+      </c>
+      <c r="C6" s="28" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D6" s="29" t="n">
+        <v>4</v>
+      </c>
+      <c r="E6" s="30" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="F6" s="30">
+        <f>D6*E6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="31" t="inlineStr">
+        <is>
+          <t>Batidora industrial</t>
+        </is>
+      </c>
+      <c r="B7" s="31" t="inlineStr">
+        <is>
+          <t>Mantequilla</t>
+        </is>
+      </c>
+      <c r="C7" s="32" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D7" s="33" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" s="34" t="n">
+        <v>18</v>
+      </c>
+      <c r="F7" s="34">
+        <f>D7*E7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="27" t="inlineStr">
+        <is>
+          <t>Batidora industrial</t>
+        </is>
+      </c>
+      <c r="B8" s="27" t="inlineStr">
+        <is>
+          <t>Huevos</t>
+        </is>
+      </c>
+      <c r="C8" s="28" t="inlineStr">
+        <is>
+          <t>docena</t>
+        </is>
+      </c>
+      <c r="D8" s="29" t="n">
+        <v>3</v>
+      </c>
+      <c r="E8" s="30" t="n">
+        <v>7</v>
+      </c>
+      <c r="F8" s="30">
+        <f>D8*E8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="31" t="inlineStr">
+        <is>
+          <t>Cocina industrial</t>
+        </is>
+      </c>
+      <c r="B9" s="31" t="inlineStr">
+        <is>
+          <t>Aceite vegetal</t>
+        </is>
+      </c>
+      <c r="C9" s="32" t="inlineStr">
+        <is>
+          <t>litro</t>
+        </is>
+      </c>
+      <c r="D9" s="33" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" s="34" t="n">
+        <v>8</v>
+      </c>
+      <c r="F9" s="34">
+        <f>D9*E9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="27" t="inlineStr">
+        <is>
+          <t>Cocina industrial</t>
+        </is>
+      </c>
+      <c r="B10" s="27" t="inlineStr">
+        <is>
+          <t>Sal fina</t>
+        </is>
+      </c>
+      <c r="C10" s="28" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D10" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="30" t="n">
+        <v>2</v>
+      </c>
+      <c r="F10" s="30">
+        <f>D10*E10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="31" t="inlineStr">
+        <is>
+          <t>Cocina industrial</t>
+        </is>
+      </c>
+      <c r="B11" s="31" t="inlineStr">
+        <is>
+          <t>Especias básicas (kit)</t>
+        </is>
+      </c>
+      <c r="C11" s="32" t="inlineStr">
+        <is>
+          <t>kit</t>
+        </is>
+      </c>
+      <c r="D11" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="34" t="n">
+        <v>25</v>
+      </c>
+      <c r="F11" s="34">
+        <f>D11*E11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="27" t="inlineStr">
+        <is>
+          <t>Selladora/envasadora</t>
+        </is>
+      </c>
+      <c r="B12" s="27" t="inlineStr">
+        <is>
+          <t>Bolsas de sellado 20x30cm</t>
+        </is>
+      </c>
+      <c r="C12" s="28" t="inlineStr">
+        <is>
+          <t>paquete x100</t>
+        </is>
+      </c>
+      <c r="D12" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="30" t="n">
+        <v>28</v>
+      </c>
+      <c r="F12" s="30">
+        <f>D12*E12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="31" t="inlineStr">
+        <is>
+          <t>Selladora/envasadora</t>
+        </is>
+      </c>
+      <c r="B13" s="31" t="inlineStr">
+        <is>
+          <t>Etiquetas adhesivas</t>
+        </is>
+      </c>
+      <c r="C13" s="32" t="inlineStr">
+        <is>
+          <t>rollo x500</t>
+        </is>
+      </c>
+      <c r="D13" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="34" t="n">
+        <v>15</v>
+      </c>
+      <c r="F13" s="34">
+        <f>D13*E13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="27" t="inlineStr">
+        <is>
+          <t>Mesas de trabajo</t>
+        </is>
+      </c>
+      <c r="B14" s="27" t="inlineStr">
+        <is>
+          <t>Guantes descartables</t>
+        </is>
+      </c>
+      <c r="C14" s="28" t="inlineStr">
+        <is>
+          <t>caja x100</t>
+        </is>
+      </c>
+      <c r="D14" s="29" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E14" s="30" t="n">
+        <v>18</v>
+      </c>
+      <c r="F14" s="30">
+        <f>D14*E14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="31" t="inlineStr">
+        <is>
+          <t>Mesas de trabajo</t>
+        </is>
+      </c>
+      <c r="B15" s="31" t="inlineStr">
+        <is>
+          <t>Gorros descartables</t>
+        </is>
+      </c>
+      <c r="C15" s="32" t="inlineStr">
+        <is>
+          <t>paquete x100</t>
+        </is>
+      </c>
+      <c r="D15" s="33" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E15" s="34" t="n">
+        <v>12</v>
+      </c>
+      <c r="F15" s="34">
+        <f>D15*E15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="27" t="inlineStr">
+        <is>
+          <t>Mesas de trabajo</t>
+        </is>
+      </c>
+      <c r="B16" s="27" t="inlineStr">
+        <is>
+          <t>Mascarillas</t>
+        </is>
+      </c>
+      <c r="C16" s="28" t="inlineStr">
+        <is>
+          <t>paquete x50</t>
+        </is>
+      </c>
+      <c r="D16" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="30" t="n">
+        <v>12</v>
+      </c>
+      <c r="F16" s="30">
+        <f>D16*E16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="35" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B17" s="35" t="inlineStr">
+        <is>
+          <t>Cocina y Repostería</t>
+        </is>
+      </c>
+      <c r="C17" s="36" t="n"/>
+      <c r="D17" s="36" t="n"/>
+      <c r="E17" s="36" t="n"/>
+      <c r="F17" s="37">
+        <f>SUM(F4:F16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="25" t="inlineStr">
+        <is>
+          <t>COMPUTACIÓN E INFORMÁTICA</t>
+        </is>
+      </c>
+      <c r="B19" s="25" t="n"/>
+      <c r="C19" s="25" t="n"/>
+      <c r="D19" s="25" t="n"/>
+      <c r="E19" s="25" t="n"/>
+      <c r="F19" s="25" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="26" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+      <c r="B20" s="26" t="inlineStr">
+        <is>
+          <t>Consumible</t>
+        </is>
+      </c>
+      <c r="C20" s="26" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="D20" s="26" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="E20" s="26" t="inlineStr">
+        <is>
+          <t>Precio Unit. (S/.)</t>
+        </is>
+      </c>
+      <c r="F20" s="26" t="inlineStr">
+        <is>
+          <t>Subtotal</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="27" t="inlineStr">
+        <is>
+          <t>PCs / Laptops</t>
+        </is>
+      </c>
+      <c r="B21" s="27" t="inlineStr">
+        <is>
+          <t>Pasta térmica</t>
+        </is>
+      </c>
+      <c r="C21" s="28" t="inlineStr">
+        <is>
+          <t>tubo 100g</t>
+        </is>
+      </c>
+      <c r="D21" s="29" t="n">
+        <v>3</v>
+      </c>
+      <c r="E21" s="30" t="n">
+        <v>18</v>
+      </c>
+      <c r="F21" s="30">
+        <f>D21*E21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="31" t="inlineStr">
+        <is>
+          <t>PCs / Laptops</t>
+        </is>
+      </c>
+      <c r="B22" s="31" t="inlineStr">
+        <is>
+          <t>Alcohol isopropílico 99%</t>
+        </is>
+      </c>
+      <c r="C22" s="32" t="inlineStr">
+        <is>
+          <t>frasco 250ml</t>
+        </is>
+      </c>
+      <c r="D22" s="33" t="n">
+        <v>2</v>
+      </c>
+      <c r="E22" s="34" t="n">
+        <v>12</v>
+      </c>
+      <c r="F22" s="34">
+        <f>D22*E22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="27" t="inlineStr">
+        <is>
+          <t>Switch / Router</t>
+        </is>
+      </c>
+      <c r="B23" s="27" t="inlineStr">
+        <is>
+          <t>Cable UTP Cat6</t>
+        </is>
+      </c>
+      <c r="C23" s="28" t="inlineStr">
+        <is>
+          <t>metro</t>
+        </is>
+      </c>
+      <c r="D23" s="29" t="n">
+        <v>20</v>
+      </c>
+      <c r="E23" s="30" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F23" s="30">
+        <f>D23*E23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="31" t="inlineStr">
+        <is>
+          <t>Switch / Router</t>
+        </is>
+      </c>
+      <c r="B24" s="31" t="inlineStr">
+        <is>
+          <t>Conectores RJ45 Cat6</t>
+        </is>
+      </c>
+      <c r="C24" s="32" t="inlineStr">
+        <is>
+          <t>bolsa x100</t>
+        </is>
+      </c>
+      <c r="D24" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="34" t="n">
+        <v>35</v>
+      </c>
+      <c r="F24" s="34">
+        <f>D24*E24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="27" t="inlineStr">
+        <is>
+          <t>Switch / Router</t>
+        </is>
+      </c>
+      <c r="B25" s="27" t="inlineStr">
+        <is>
+          <t>Ponchadora RJ45 (reemplazo cuchilla)</t>
+        </is>
+      </c>
+      <c r="C25" s="28" t="inlineStr">
+        <is>
+          <t>pieza</t>
+        </is>
+      </c>
+      <c r="D25" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" s="30" t="n">
+        <v>15</v>
+      </c>
+      <c r="F25" s="30">
+        <f>D25*E25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="31" t="inlineStr">
+        <is>
+          <t>Impresora</t>
+        </is>
+      </c>
+      <c r="B26" s="31" t="inlineStr">
+        <is>
+          <t>Papel bond A4</t>
+        </is>
+      </c>
+      <c r="C26" s="32" t="inlineStr">
+        <is>
+          <t>resma 500h</t>
+        </is>
+      </c>
+      <c r="D26" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" s="34" t="n">
+        <v>22</v>
+      </c>
+      <c r="F26" s="34">
+        <f>D26*E26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="27" t="inlineStr">
+        <is>
+          <t>Herramientas ensamblaje</t>
+        </is>
+      </c>
+      <c r="B27" s="27" t="inlineStr">
+        <is>
+          <t>Pulsera antiestática</t>
+        </is>
+      </c>
+      <c r="C27" s="28" t="inlineStr">
+        <is>
+          <t>unidad</t>
+        </is>
+      </c>
+      <c r="D27" s="29" t="n">
+        <v>5</v>
+      </c>
+      <c r="E27" s="30" t="n">
+        <v>12</v>
+      </c>
+      <c r="F27" s="30">
+        <f>D27*E27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="31" t="inlineStr">
+        <is>
+          <t>Herramientas ensamblaje</t>
+        </is>
+      </c>
+      <c r="B28" s="31" t="inlineStr">
+        <is>
+          <t>Bridas surtidas</t>
+        </is>
+      </c>
+      <c r="C28" s="32" t="inlineStr">
+        <is>
+          <t>paquete x100</t>
+        </is>
+      </c>
+      <c r="D28" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" s="34" t="n">
+        <v>8</v>
+      </c>
+      <c r="F28" s="34">
+        <f>D28*E28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="35" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B29" s="35" t="inlineStr">
+        <is>
+          <t>Computación e Informática</t>
+        </is>
+      </c>
+      <c r="C29" s="36" t="n"/>
+      <c r="D29" s="36" t="n"/>
+      <c r="E29" s="36" t="n"/>
+      <c r="F29" s="37">
+        <f>SUM(F21:F28)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" ht="22" customHeight="1">
+      <c r="A31" s="25" t="inlineStr">
+        <is>
+          <t>CONSTRUCCIONES METÁLICAS</t>
+        </is>
+      </c>
+      <c r="B31" s="25" t="n"/>
+      <c r="C31" s="25" t="n"/>
+      <c r="D31" s="25" t="n"/>
+      <c r="E31" s="25" t="n"/>
+      <c r="F31" s="25" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="26" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+      <c r="B32" s="26" t="inlineStr">
+        <is>
+          <t>Consumible</t>
+        </is>
+      </c>
+      <c r="C32" s="26" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="D32" s="26" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="E32" s="26" t="inlineStr">
+        <is>
+          <t>Precio Unit. (S/.)</t>
+        </is>
+      </c>
+      <c r="F32" s="26" t="inlineStr">
+        <is>
+          <t>Subtotal</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="27" t="inlineStr">
+        <is>
+          <t>Soldadora MIG/MAG</t>
+        </is>
+      </c>
+      <c r="B33" s="27" t="inlineStr">
+        <is>
+          <t>Alambre MIG 0.8mm</t>
+        </is>
+      </c>
+      <c r="C33" s="28" t="inlineStr">
+        <is>
+          <t>rollo 5kg</t>
+        </is>
+      </c>
+      <c r="D33" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" s="30" t="n">
+        <v>120</v>
+      </c>
+      <c r="F33" s="30">
+        <f>D33*E33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="31" t="inlineStr">
+        <is>
+          <t>Soldadora MIG/MAG</t>
+        </is>
+      </c>
+      <c r="B34" s="31" t="inlineStr">
+        <is>
+          <t>Gas CO2 (mezcla)</t>
+        </is>
+      </c>
+      <c r="C34" s="32" t="inlineStr">
+        <is>
+          <t>balón 10kg</t>
+        </is>
+      </c>
+      <c r="D34" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" s="34" t="n">
+        <v>85</v>
+      </c>
+      <c r="F34" s="34">
+        <f>D34*E34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="27" t="inlineStr">
+        <is>
+          <t>Soldadora eléctrica (SMAW)</t>
+        </is>
+      </c>
+      <c r="B35" s="27" t="inlineStr">
+        <is>
+          <t>Electrodos 6011 3.2mm</t>
+        </is>
+      </c>
+      <c r="C35" s="28" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D35" s="29" t="n">
+        <v>4</v>
+      </c>
+      <c r="E35" s="30" t="n">
+        <v>12</v>
+      </c>
+      <c r="F35" s="30">
+        <f>D35*E35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="31" t="inlineStr">
+        <is>
+          <t>Soldadora eléctrica (SMAW)</t>
+        </is>
+      </c>
+      <c r="B36" s="31" t="inlineStr">
+        <is>
+          <t>Electrodos 7018 3.2mm</t>
+        </is>
+      </c>
+      <c r="C36" s="32" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D36" s="33" t="n">
+        <v>4</v>
+      </c>
+      <c r="E36" s="34" t="n">
+        <v>14</v>
+      </c>
+      <c r="F36" s="34">
+        <f>D36*E36</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="27" t="inlineStr">
+        <is>
+          <t>Soldadora TIG</t>
+        </is>
+      </c>
+      <c r="B37" s="27" t="inlineStr">
+        <is>
+          <t>Varillas TIG ER70S 2.4mm</t>
+        </is>
+      </c>
+      <c r="C37" s="28" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D37" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E37" s="30" t="n">
+        <v>45</v>
+      </c>
+      <c r="F37" s="30">
+        <f>D37*E37</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="31" t="inlineStr">
+        <is>
+          <t>Soldadora TIG</t>
+        </is>
+      </c>
+      <c r="B38" s="31" t="inlineStr">
+        <is>
+          <t>Gas argón</t>
+        </is>
+      </c>
+      <c r="C38" s="32" t="inlineStr">
+        <is>
+          <t>balón 10m³</t>
+        </is>
+      </c>
+      <c r="D38" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="E38" s="34" t="n">
+        <v>120</v>
+      </c>
+      <c r="F38" s="34">
+        <f>D38*E38</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="27" t="inlineStr">
+        <is>
+          <t>Cortadora plasma</t>
+        </is>
+      </c>
+      <c r="B39" s="27" t="inlineStr">
+        <is>
+          <t>Electrodos de plasma</t>
+        </is>
+      </c>
+      <c r="C39" s="28" t="inlineStr">
+        <is>
+          <t>paquete x5</t>
+        </is>
+      </c>
+      <c r="D39" s="29" t="n">
+        <v>2</v>
+      </c>
+      <c r="E39" s="30" t="n">
+        <v>35</v>
+      </c>
+      <c r="F39" s="30">
+        <f>D39*E39</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="31" t="inlineStr">
+        <is>
+          <t>Cortadora plasma</t>
+        </is>
+      </c>
+      <c r="B40" s="31" t="inlineStr">
+        <is>
+          <t>Toberas de plasma</t>
+        </is>
+      </c>
+      <c r="C40" s="32" t="inlineStr">
+        <is>
+          <t>paquete x5</t>
+        </is>
+      </c>
+      <c r="D40" s="33" t="n">
+        <v>2</v>
+      </c>
+      <c r="E40" s="34" t="n">
+        <v>40</v>
+      </c>
+      <c r="F40" s="34">
+        <f>D40*E40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="27" t="inlineStr">
+        <is>
+          <t>Amoladora angular</t>
+        </is>
+      </c>
+      <c r="B41" s="27" t="inlineStr">
+        <is>
+          <t>Disco de corte 4.5"</t>
+        </is>
+      </c>
+      <c r="C41" s="28" t="inlineStr">
+        <is>
+          <t>paquete x10</t>
+        </is>
+      </c>
+      <c r="D41" s="29" t="n">
+        <v>2</v>
+      </c>
+      <c r="E41" s="30" t="n">
+        <v>35</v>
+      </c>
+      <c r="F41" s="30">
+        <f>D41*E41</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="31" t="inlineStr">
+        <is>
+          <t>Amoladora angular</t>
+        </is>
+      </c>
+      <c r="B42" s="31" t="inlineStr">
+        <is>
+          <t>Disco de desbaste 4.5"</t>
+        </is>
+      </c>
+      <c r="C42" s="32" t="inlineStr">
+        <is>
+          <t>paquete x5</t>
+        </is>
+      </c>
+      <c r="D42" s="33" t="n">
+        <v>2</v>
+      </c>
+      <c r="E42" s="34" t="n">
+        <v>28</v>
+      </c>
+      <c r="F42" s="34">
+        <f>D42*E42</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="27" t="inlineStr">
+        <is>
+          <t>Taladro de banco</t>
+        </is>
+      </c>
+      <c r="B43" s="27" t="inlineStr">
+        <is>
+          <t>Brocas HSS surtido</t>
+        </is>
+      </c>
+      <c r="C43" s="28" t="inlineStr">
+        <is>
+          <t>set</t>
+        </is>
+      </c>
+      <c r="D43" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E43" s="30" t="n">
+        <v>45</v>
+      </c>
+      <c r="F43" s="30">
+        <f>D43*E43</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="31" t="inlineStr">
+        <is>
+          <t>Material de práctica</t>
+        </is>
+      </c>
+      <c r="B44" s="31" t="inlineStr">
+        <is>
+          <t>Platina/ángulo acero</t>
+        </is>
+      </c>
+      <c r="C44" s="32" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D44" s="33" t="n">
+        <v>20</v>
+      </c>
+      <c r="E44" s="34" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="F44" s="34">
+        <f>D44*E44</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45" ht="20" customHeight="1">
+      <c r="A45" s="35" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B45" s="35" t="inlineStr">
+        <is>
+          <t>Construcciones Metálicas</t>
+        </is>
+      </c>
+      <c r="C45" s="36" t="n"/>
+      <c r="D45" s="36" t="n"/>
+      <c r="E45" s="36" t="n"/>
+      <c r="F45" s="37">
+        <f>SUM(F33:F44)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47" ht="22" customHeight="1">
+      <c r="A47" s="25" t="inlineStr">
+        <is>
+          <t>EBANISTERÍA</t>
+        </is>
+      </c>
+      <c r="B47" s="25" t="n"/>
+      <c r="C47" s="25" t="n"/>
+      <c r="D47" s="25" t="n"/>
+      <c r="E47" s="25" t="n"/>
+      <c r="F47" s="25" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="26" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+      <c r="B48" s="26" t="inlineStr">
+        <is>
+          <t>Consumible</t>
+        </is>
+      </c>
+      <c r="C48" s="26" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="D48" s="26" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="E48" s="26" t="inlineStr">
+        <is>
+          <t>Precio Unit. (S/.)</t>
+        </is>
+      </c>
+      <c r="F48" s="26" t="inlineStr">
+        <is>
+          <t>Subtotal</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="27" t="inlineStr">
+        <is>
+          <t>Sierra circular de mesa</t>
+        </is>
+      </c>
+      <c r="B49" s="27" t="inlineStr">
+        <is>
+          <t>Hoja sierra 60T 10"</t>
+        </is>
+      </c>
+      <c r="C49" s="28" t="inlineStr">
+        <is>
+          <t>unidad</t>
+        </is>
+      </c>
+      <c r="D49" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E49" s="30" t="n">
+        <v>65</v>
+      </c>
+      <c r="F49" s="30">
+        <f>D49*E49</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="31" t="inlineStr">
+        <is>
+          <t>Sierra circular de mesa</t>
+        </is>
+      </c>
+      <c r="B50" s="31" t="inlineStr">
+        <is>
+          <t>MDF 15mm 1.83x2.44m</t>
+        </is>
+      </c>
+      <c r="C50" s="32" t="inlineStr">
+        <is>
+          <t>plancha</t>
+        </is>
+      </c>
+      <c r="D50" s="33" t="n">
+        <v>3</v>
+      </c>
+      <c r="E50" s="34" t="n">
+        <v>78</v>
+      </c>
+      <c r="F50" s="34">
+        <f>D50*E50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="27" t="inlineStr">
+        <is>
+          <t>Sierra de cinta</t>
+        </is>
+      </c>
+      <c r="B51" s="27" t="inlineStr">
+        <is>
+          <t>Hoja de banda (reemplazo)</t>
+        </is>
+      </c>
+      <c r="C51" s="28" t="inlineStr">
+        <is>
+          <t>unidad</t>
+        </is>
+      </c>
+      <c r="D51" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E51" s="30" t="n">
+        <v>68</v>
+      </c>
+      <c r="F51" s="30">
+        <f>D51*E51</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="31" t="inlineStr">
+        <is>
+          <t>Router / CNC</t>
+        </is>
+      </c>
+      <c r="B52" s="31" t="inlineStr">
+        <is>
+          <t>Fresa recta 6mm carburo</t>
+        </is>
+      </c>
+      <c r="C52" s="32" t="inlineStr">
+        <is>
+          <t>unidad</t>
+        </is>
+      </c>
+      <c r="D52" s="33" t="n">
+        <v>3</v>
+      </c>
+      <c r="E52" s="34" t="n">
+        <v>38</v>
+      </c>
+      <c r="F52" s="34">
+        <f>D52*E52</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="27" t="inlineStr">
+        <is>
+          <t>Router / CNC</t>
+        </is>
+      </c>
+      <c r="B53" s="27" t="inlineStr">
+        <is>
+          <t>Fresa de perfil 1/4"</t>
+        </is>
+      </c>
+      <c r="C53" s="28" t="inlineStr">
+        <is>
+          <t>unidad</t>
+        </is>
+      </c>
+      <c r="D53" s="29" t="n">
+        <v>2</v>
+      </c>
+      <c r="E53" s="30" t="n">
+        <v>42</v>
+      </c>
+      <c r="F53" s="30">
+        <f>D53*E53</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="31" t="inlineStr">
+        <is>
+          <t>Lijadora orbital</t>
+        </is>
+      </c>
+      <c r="B54" s="31" t="inlineStr">
+        <is>
+          <t>Disco lija 80 5"</t>
+        </is>
+      </c>
+      <c r="C54" s="32" t="inlineStr">
+        <is>
+          <t>paquete x20</t>
+        </is>
+      </c>
+      <c r="D54" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="E54" s="34" t="n">
+        <v>22</v>
+      </c>
+      <c r="F54" s="34">
+        <f>D54*E54</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="27" t="inlineStr">
+        <is>
+          <t>Lijadora orbital</t>
+        </is>
+      </c>
+      <c r="B55" s="27" t="inlineStr">
+        <is>
+          <t>Disco lija 120 5"</t>
+        </is>
+      </c>
+      <c r="C55" s="28" t="inlineStr">
+        <is>
+          <t>paquete x20</t>
+        </is>
+      </c>
+      <c r="D55" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E55" s="30" t="n">
+        <v>22</v>
+      </c>
+      <c r="F55" s="30">
+        <f>D55*E55</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="31" t="inlineStr">
+        <is>
+          <t>Lijadora orbital</t>
+        </is>
+      </c>
+      <c r="B56" s="31" t="inlineStr">
+        <is>
+          <t>Disco lija 220 5"</t>
+        </is>
+      </c>
+      <c r="C56" s="32" t="inlineStr">
+        <is>
+          <t>paquete x20</t>
+        </is>
+      </c>
+      <c r="D56" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="E56" s="34" t="n">
+        <v>25</v>
+      </c>
+      <c r="F56" s="34">
+        <f>D56*E56</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="27" t="inlineStr">
+        <is>
+          <t>Torno de madera</t>
+        </is>
+      </c>
+      <c r="B57" s="27" t="inlineStr">
+        <is>
+          <t>Lija para torno (rollo)</t>
+        </is>
+      </c>
+      <c r="C57" s="28" t="inlineStr">
+        <is>
+          <t>metro</t>
+        </is>
+      </c>
+      <c r="D57" s="29" t="n">
+        <v>5</v>
+      </c>
+      <c r="E57" s="30" t="n">
+        <v>4</v>
+      </c>
+      <c r="F57" s="30">
+        <f>D57*E57</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="31" t="inlineStr">
+        <is>
+          <t>Compresor + pistola</t>
+        </is>
+      </c>
+      <c r="B58" s="31" t="inlineStr">
+        <is>
+          <t>Sellador madera</t>
+        </is>
+      </c>
+      <c r="C58" s="32" t="inlineStr">
+        <is>
+          <t>litro</t>
+        </is>
+      </c>
+      <c r="D58" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="E58" s="34" t="n">
+        <v>28</v>
+      </c>
+      <c r="F58" s="34">
+        <f>D58*E58</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="27" t="inlineStr">
+        <is>
+          <t>Compresor + pistola</t>
+        </is>
+      </c>
+      <c r="B59" s="27" t="inlineStr">
+        <is>
+          <t>Barniz brillante</t>
+        </is>
+      </c>
+      <c r="C59" s="28" t="inlineStr">
+        <is>
+          <t>litro</t>
+        </is>
+      </c>
+      <c r="D59" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E59" s="30" t="n">
+        <v>32</v>
+      </c>
+      <c r="F59" s="30">
+        <f>D59*E59</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="31" t="inlineStr">
+        <is>
+          <t>Compresor + pistola</t>
+        </is>
+      </c>
+      <c r="B60" s="31" t="inlineStr">
+        <is>
+          <t>Thinner</t>
+        </is>
+      </c>
+      <c r="C60" s="32" t="inlineStr">
+        <is>
+          <t>litro</t>
+        </is>
+      </c>
+      <c r="D60" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="E60" s="34" t="n">
+        <v>12</v>
+      </c>
+      <c r="F60" s="34">
+        <f>D60*E60</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="27" t="inlineStr">
+        <is>
+          <t>Material de práctica</t>
+        </is>
+      </c>
+      <c r="B61" s="27" t="inlineStr">
+        <is>
+          <t>Tablas tornillo 1"x4"x8'</t>
+        </is>
+      </c>
+      <c r="C61" s="28" t="inlineStr">
+        <is>
+          <t>unidad</t>
+        </is>
+      </c>
+      <c r="D61" s="29" t="n">
+        <v>8</v>
+      </c>
+      <c r="E61" s="30" t="n">
+        <v>18</v>
+      </c>
+      <c r="F61" s="30">
+        <f>D61*E61</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62" ht="20" customHeight="1">
+      <c r="A62" s="35" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B62" s="35" t="inlineStr">
+        <is>
+          <t>Ebanistería</t>
+        </is>
+      </c>
+      <c r="C62" s="36" t="n"/>
+      <c r="D62" s="36" t="n"/>
+      <c r="E62" s="36" t="n"/>
+      <c r="F62" s="37">
+        <f>SUM(F49:F61)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64" ht="22" customHeight="1">
+      <c r="A64" s="25" t="inlineStr">
+        <is>
+          <t>ELECTRICIDAD</t>
+        </is>
+      </c>
+      <c r="B64" s="25" t="n"/>
+      <c r="C64" s="25" t="n"/>
+      <c r="D64" s="25" t="n"/>
+      <c r="E64" s="25" t="n"/>
+      <c r="F64" s="25" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="26" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+      <c r="B65" s="26" t="inlineStr">
+        <is>
+          <t>Consumible</t>
+        </is>
+      </c>
+      <c r="C65" s="26" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="D65" s="26" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="E65" s="26" t="inlineStr">
+        <is>
+          <t>Precio Unit. (S/.)</t>
+        </is>
+      </c>
+      <c r="F65" s="26" t="inlineStr">
+        <is>
+          <t>Subtotal</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="27" t="inlineStr">
+        <is>
+          <t>Tablero de prácticas</t>
+        </is>
+      </c>
+      <c r="B66" s="27" t="inlineStr">
+        <is>
+          <t>Cable THW 14AWG (rojo)</t>
+        </is>
+      </c>
+      <c r="C66" s="28" t="inlineStr">
+        <is>
+          <t>metro</t>
+        </is>
+      </c>
+      <c r="D66" s="29" t="n">
+        <v>20</v>
+      </c>
+      <c r="E66" s="30" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="F66" s="30">
+        <f>D66*E66</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="31" t="inlineStr">
+        <is>
+          <t>Tablero de prácticas</t>
+        </is>
+      </c>
+      <c r="B67" s="31" t="inlineStr">
+        <is>
+          <t>Cable THW 14AWG (negro)</t>
+        </is>
+      </c>
+      <c r="C67" s="32" t="inlineStr">
+        <is>
+          <t>metro</t>
+        </is>
+      </c>
+      <c r="D67" s="33" t="n">
+        <v>20</v>
+      </c>
+      <c r="E67" s="34" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="F67" s="34">
+        <f>D67*E67</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="27" t="inlineStr">
+        <is>
+          <t>Tablero de prácticas</t>
+        </is>
+      </c>
+      <c r="B68" s="27" t="inlineStr">
+        <is>
+          <t>Cable THW 14AWG (verde)</t>
+        </is>
+      </c>
+      <c r="C68" s="28" t="inlineStr">
+        <is>
+          <t>metro</t>
+        </is>
+      </c>
+      <c r="D68" s="29" t="n">
+        <v>10</v>
+      </c>
+      <c r="E68" s="30" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="F68" s="30">
+        <f>D68*E68</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="31" t="inlineStr">
+        <is>
+          <t>Tablero de prácticas</t>
+        </is>
+      </c>
+      <c r="B69" s="31" t="inlineStr">
+        <is>
+          <t>Terminales preaislados surtido</t>
+        </is>
+      </c>
+      <c r="C69" s="32" t="inlineStr">
+        <is>
+          <t>bolsa x100</t>
+        </is>
+      </c>
+      <c r="D69" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="E69" s="34" t="n">
+        <v>28</v>
+      </c>
+      <c r="F69" s="34">
+        <f>D69*E69</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="27" t="inlineStr">
+        <is>
+          <t>Módulo automatización</t>
+        </is>
+      </c>
+      <c r="B70" s="27" t="inlineStr">
+        <is>
+          <t>Relé 24VDC con base</t>
+        </is>
+      </c>
+      <c r="C70" s="28" t="inlineStr">
+        <is>
+          <t>unidad</t>
+        </is>
+      </c>
+      <c r="D70" s="29" t="n">
+        <v>5</v>
+      </c>
+      <c r="E70" s="30" t="n">
+        <v>12</v>
+      </c>
+      <c r="F70" s="30">
+        <f>D70*E70</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="31" t="inlineStr">
+        <is>
+          <t>Módulo automatización</t>
+        </is>
+      </c>
+      <c r="B71" s="31" t="inlineStr">
+        <is>
+          <t>Contactor LC1-D09</t>
+        </is>
+      </c>
+      <c r="C71" s="32" t="inlineStr">
+        <is>
+          <t>unidad</t>
+        </is>
+      </c>
+      <c r="D71" s="33" t="n">
+        <v>3</v>
+      </c>
+      <c r="E71" s="34" t="n">
+        <v>42</v>
+      </c>
+      <c r="F71" s="34">
+        <f>D71*E71</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="27" t="inlineStr">
+        <is>
+          <t>Módulo automatización</t>
+        </is>
+      </c>
+      <c r="B72" s="27" t="inlineStr">
+        <is>
+          <t>Cinta aislante 19mm</t>
+        </is>
+      </c>
+      <c r="C72" s="28" t="inlineStr">
+        <is>
+          <t>rollo</t>
+        </is>
+      </c>
+      <c r="D72" s="29" t="n">
+        <v>5</v>
+      </c>
+      <c r="E72" s="30" t="n">
+        <v>4</v>
+      </c>
+      <c r="F72" s="30">
+        <f>D72*E72</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="31" t="inlineStr">
+        <is>
+          <t>Instalaciones práctica</t>
+        </is>
+      </c>
+      <c r="B73" s="31" t="inlineStr">
+        <is>
+          <t>Tubería PVC 3/4"</t>
+        </is>
+      </c>
+      <c r="C73" s="32" t="inlineStr">
+        <is>
+          <t>metro</t>
+        </is>
+      </c>
+      <c r="D73" s="33" t="n">
+        <v>10</v>
+      </c>
+      <c r="E73" s="34" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="F73" s="34">
+        <f>D73*E73</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="27" t="inlineStr">
+        <is>
+          <t>Instalaciones práctica</t>
+        </is>
+      </c>
+      <c r="B74" s="27" t="inlineStr">
+        <is>
+          <t>Curvas PVC 3/4"</t>
+        </is>
+      </c>
+      <c r="C74" s="28" t="inlineStr">
+        <is>
+          <t>unidad</t>
+        </is>
+      </c>
+      <c r="D74" s="29" t="n">
+        <v>10</v>
+      </c>
+      <c r="E74" s="30" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F74" s="30">
+        <f>D74*E74</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="31" t="inlineStr">
+        <is>
+          <t>Instalaciones práctica</t>
+        </is>
+      </c>
+      <c r="B75" s="31" t="inlineStr">
+        <is>
+          <t>Cajas de pase 100x100</t>
+        </is>
+      </c>
+      <c r="C75" s="32" t="inlineStr">
+        <is>
+          <t>unidad</t>
+        </is>
+      </c>
+      <c r="D75" s="33" t="n">
+        <v>5</v>
+      </c>
+      <c r="E75" s="34" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="F75" s="34">
+        <f>D75*E75</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="27" t="inlineStr">
+        <is>
+          <t>Equipo de medición</t>
+        </is>
+      </c>
+      <c r="B76" s="27" t="inlineStr">
+        <is>
+          <t>Fusibles surtido</t>
+        </is>
+      </c>
+      <c r="C76" s="28" t="inlineStr">
+        <is>
+          <t>paquete x20</t>
+        </is>
+      </c>
+      <c r="D76" s="29" t="n">
+        <v>2</v>
+      </c>
+      <c r="E76" s="30" t="n">
+        <v>12</v>
+      </c>
+      <c r="F76" s="30">
+        <f>D76*E76</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77" ht="20" customHeight="1">
+      <c r="A77" s="35" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B77" s="35" t="inlineStr">
+        <is>
+          <t>Electricidad</t>
+        </is>
+      </c>
+      <c r="C77" s="36" t="n"/>
+      <c r="D77" s="36" t="n"/>
+      <c r="E77" s="36" t="n"/>
+      <c r="F77" s="37">
+        <f>SUM(F66:F76)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79" ht="22" customHeight="1">
+      <c r="A79" s="25" t="inlineStr">
+        <is>
+          <t>ELECTRÓNICA</t>
+        </is>
+      </c>
+      <c r="B79" s="25" t="n"/>
+      <c r="C79" s="25" t="n"/>
+      <c r="D79" s="25" t="n"/>
+      <c r="E79" s="25" t="n"/>
+      <c r="F79" s="25" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="26" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+      <c r="B80" s="26" t="inlineStr">
+        <is>
+          <t>Consumible</t>
+        </is>
+      </c>
+      <c r="C80" s="26" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="D80" s="26" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="E80" s="26" t="inlineStr">
+        <is>
+          <t>Precio Unit. (S/.)</t>
+        </is>
+      </c>
+      <c r="F80" s="26" t="inlineStr">
+        <is>
+          <t>Subtotal</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="27" t="inlineStr">
+        <is>
+          <t>Estación de soldadura</t>
+        </is>
+      </c>
+      <c r="B81" s="27" t="inlineStr">
+        <is>
+          <t>Estaño 60/40 1mm</t>
+        </is>
+      </c>
+      <c r="C81" s="28" t="inlineStr">
+        <is>
+          <t>rollo 250g</t>
+        </is>
+      </c>
+      <c r="D81" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E81" s="30" t="n">
+        <v>32</v>
+      </c>
+      <c r="F81" s="30">
+        <f>D81*E81</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="31" t="inlineStr">
+        <is>
+          <t>Estación de soldadura</t>
+        </is>
+      </c>
+      <c r="B82" s="31" t="inlineStr">
+        <is>
+          <t>Flux líquido</t>
+        </is>
+      </c>
+      <c r="C82" s="32" t="inlineStr">
+        <is>
+          <t>frasco 50ml</t>
+        </is>
+      </c>
+      <c r="D82" s="33" t="n">
+        <v>2</v>
+      </c>
+      <c r="E82" s="34" t="n">
+        <v>18</v>
+      </c>
+      <c r="F82" s="34">
+        <f>D82*E82</f>
+        <v/>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="27" t="inlineStr">
+        <is>
+          <t>Estación de soldadura</t>
+        </is>
+      </c>
+      <c r="B83" s="27" t="inlineStr">
+        <is>
+          <t>Esponja de limpieza</t>
+        </is>
+      </c>
+      <c r="C83" s="28" t="inlineStr">
+        <is>
+          <t>unidad</t>
+        </is>
+      </c>
+      <c r="D83" s="29" t="n">
+        <v>3</v>
+      </c>
+      <c r="E83" s="30" t="n">
+        <v>5</v>
+      </c>
+      <c r="F83" s="30">
+        <f>D83*E83</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="31" t="inlineStr">
+        <is>
+          <t>Estación de aire (SMD)</t>
+        </is>
+      </c>
+      <c r="B84" s="31" t="inlineStr">
+        <is>
+          <t>Pasta soldadora SMD</t>
+        </is>
+      </c>
+      <c r="C84" s="32" t="inlineStr">
+        <is>
+          <t>jeringa 50g</t>
+        </is>
+      </c>
+      <c r="D84" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="E84" s="34" t="n">
+        <v>38</v>
+      </c>
+      <c r="F84" s="34">
+        <f>D84*E84</f>
+        <v/>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="27" t="inlineStr">
+        <is>
+          <t>Estación de aire (SMD)</t>
+        </is>
+      </c>
+      <c r="B85" s="27" t="inlineStr">
+        <is>
+          <t>Mecha desoldar 2.5mm</t>
+        </is>
+      </c>
+      <c r="C85" s="28" t="inlineStr">
+        <is>
+          <t>rollo x3</t>
+        </is>
+      </c>
+      <c r="D85" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E85" s="30" t="n">
+        <v>20</v>
+      </c>
+      <c r="F85" s="30">
+        <f>D85*E85</f>
+        <v/>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="31" t="inlineStr">
+        <is>
+          <t>Protoboard / PCB</t>
+        </is>
+      </c>
+      <c r="B86" s="31" t="inlineStr">
+        <is>
+          <t>PCB virgen fibra 10x15cm</t>
+        </is>
+      </c>
+      <c r="C86" s="32" t="inlineStr">
+        <is>
+          <t>unidad</t>
+        </is>
+      </c>
+      <c r="D86" s="33" t="n">
+        <v>10</v>
+      </c>
+      <c r="E86" s="34" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="F86" s="34">
+        <f>D86*E86</f>
+        <v/>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="27" t="inlineStr">
+        <is>
+          <t>Protoboard / PCB</t>
+        </is>
+      </c>
+      <c r="B87" s="27" t="inlineStr">
+        <is>
+          <t>Resistencias surtido</t>
+        </is>
+      </c>
+      <c r="C87" s="28" t="inlineStr">
+        <is>
+          <t>kit 600u</t>
+        </is>
+      </c>
+      <c r="D87" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E87" s="30" t="n">
+        <v>22</v>
+      </c>
+      <c r="F87" s="30">
+        <f>D87*E87</f>
+        <v/>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="31" t="inlineStr">
+        <is>
+          <t>Protoboard / PCB</t>
+        </is>
+      </c>
+      <c r="B88" s="31" t="inlineStr">
+        <is>
+          <t>Condensadores surtido</t>
+        </is>
+      </c>
+      <c r="C88" s="32" t="inlineStr">
+        <is>
+          <t>kit 200u</t>
+        </is>
+      </c>
+      <c r="D88" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="E88" s="34" t="n">
+        <v>28</v>
+      </c>
+      <c r="F88" s="34">
+        <f>D88*E88</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="27" t="inlineStr">
+        <is>
+          <t>Protoboard / PCB</t>
+        </is>
+      </c>
+      <c r="B89" s="27" t="inlineStr">
+        <is>
+          <t>Transistores BC547/BC557</t>
+        </is>
+      </c>
+      <c r="C89" s="28" t="inlineStr">
+        <is>
+          <t>paquete x50</t>
+        </is>
+      </c>
+      <c r="D89" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E89" s="30" t="n">
+        <v>18</v>
+      </c>
+      <c r="F89" s="30">
+        <f>D89*E89</f>
+        <v/>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="31" t="inlineStr">
+        <is>
+          <t>Protoboard / PCB</t>
+        </is>
+      </c>
+      <c r="B90" s="31" t="inlineStr">
+        <is>
+          <t>ICs básicos (555, LM358, 7805)</t>
+        </is>
+      </c>
+      <c r="C90" s="32" t="inlineStr">
+        <is>
+          <t>kit</t>
+        </is>
+      </c>
+      <c r="D90" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="E90" s="34" t="n">
+        <v>35</v>
+      </c>
+      <c r="F90" s="34">
+        <f>D90*E90</f>
+        <v/>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="27" t="inlineStr">
+        <is>
+          <t>Protoboard / PCB</t>
+        </is>
+      </c>
+      <c r="B91" s="27" t="inlineStr">
+        <is>
+          <t>Cables jumper M-M 20cm</t>
+        </is>
+      </c>
+      <c r="C91" s="28" t="inlineStr">
+        <is>
+          <t>paquete x40</t>
+        </is>
+      </c>
+      <c r="D91" s="29" t="n">
+        <v>2</v>
+      </c>
+      <c r="E91" s="30" t="n">
+        <v>12</v>
+      </c>
+      <c r="F91" s="30">
+        <f>D91*E91</f>
+        <v/>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="31" t="inlineStr">
+        <is>
+          <t>Fuente de alimentación</t>
+        </is>
+      </c>
+      <c r="B92" s="31" t="inlineStr">
+        <is>
+          <t>Cables banana-cocodrilo</t>
+        </is>
+      </c>
+      <c r="C92" s="32" t="inlineStr">
+        <is>
+          <t>par</t>
+        </is>
+      </c>
+      <c r="D92" s="33" t="n">
+        <v>4</v>
+      </c>
+      <c r="E92" s="34" t="n">
+        <v>8</v>
+      </c>
+      <c r="F92" s="34">
+        <f>D92*E92</f>
+        <v/>
+      </c>
+    </row>
+    <row r="93" ht="20" customHeight="1">
+      <c r="A93" s="35" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B93" s="35" t="inlineStr">
+        <is>
+          <t>Electrónica</t>
+        </is>
+      </c>
+      <c r="C93" s="36" t="n"/>
+      <c r="D93" s="36" t="n"/>
+      <c r="E93" s="36" t="n"/>
+      <c r="F93" s="37">
+        <f>SUM(F81:F92)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="95" ht="22" customHeight="1">
+      <c r="A95" s="25" t="inlineStr">
+        <is>
+          <t>INDUSTRIA ALIMENTARIA</t>
+        </is>
+      </c>
+      <c r="B95" s="25" t="n"/>
+      <c r="C95" s="25" t="n"/>
+      <c r="D95" s="25" t="n"/>
+      <c r="E95" s="25" t="n"/>
+      <c r="F95" s="25" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="26" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+      <c r="B96" s="26" t="inlineStr">
+        <is>
+          <t>Consumible</t>
+        </is>
+      </c>
+      <c r="C96" s="26" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="D96" s="26" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="E96" s="26" t="inlineStr">
+        <is>
+          <t>Precio Unit. (S/.)</t>
+        </is>
+      </c>
+      <c r="F96" s="26" t="inlineStr">
+        <is>
+          <t>Subtotal</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="27" t="inlineStr">
+        <is>
+          <t>Mezcladora industrial</t>
+        </is>
+      </c>
+      <c r="B97" s="27" t="inlineStr">
+        <is>
+          <t>Harina preparada</t>
+        </is>
+      </c>
+      <c r="C97" s="28" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D97" s="29" t="n">
+        <v>6</v>
+      </c>
+      <c r="E97" s="30" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="F97" s="30">
+        <f>D97*E97</f>
+        <v/>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="31" t="inlineStr">
+        <is>
+          <t>Mezcladora industrial</t>
+        </is>
+      </c>
+      <c r="B98" s="31" t="inlineStr">
+        <is>
+          <t>Azúcar blanca</t>
+        </is>
+      </c>
+      <c r="C98" s="32" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D98" s="33" t="n">
+        <v>4</v>
+      </c>
+      <c r="E98" s="34" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="F98" s="34">
+        <f>D98*E98</f>
+        <v/>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="27" t="inlineStr">
+        <is>
+          <t>Mezcladora industrial</t>
+        </is>
+      </c>
+      <c r="B99" s="27" t="inlineStr">
+        <is>
+          <t>Sal</t>
+        </is>
+      </c>
+      <c r="C99" s="28" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D99" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E99" s="30" t="n">
+        <v>2</v>
+      </c>
+      <c r="F99" s="30">
+        <f>D99*E99</f>
+        <v/>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="31" t="inlineStr">
+        <is>
+          <t>Pasteurizador</t>
+        </is>
+      </c>
+      <c r="B100" s="31" t="inlineStr">
+        <is>
+          <t>Leche fresca</t>
+        </is>
+      </c>
+      <c r="C100" s="32" t="inlineStr">
+        <is>
+          <t>litro</t>
+        </is>
+      </c>
+      <c r="D100" s="33" t="n">
+        <v>10</v>
+      </c>
+      <c r="E100" s="34" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="F100" s="34">
+        <f>D100*E100</f>
+        <v/>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="27" t="inlineStr">
+        <is>
+          <t>Pasteurizador</t>
+        </is>
+      </c>
+      <c r="B101" s="27" t="inlineStr">
+        <is>
+          <t>Envases de vidrio 250ml</t>
+        </is>
+      </c>
+      <c r="C101" s="28" t="inlineStr">
+        <is>
+          <t>unidad</t>
+        </is>
+      </c>
+      <c r="D101" s="29" t="n">
+        <v>20</v>
+      </c>
+      <c r="E101" s="30" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F101" s="30">
+        <f>D101*E101</f>
+        <v/>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="31" t="inlineStr">
+        <is>
+          <t>Selladora al vacío</t>
+        </is>
+      </c>
+      <c r="B102" s="31" t="inlineStr">
+        <is>
+          <t>Bolsas vacío 20x30cm</t>
+        </is>
+      </c>
+      <c r="C102" s="32" t="inlineStr">
+        <is>
+          <t>paquete x100</t>
+        </is>
+      </c>
+      <c r="D102" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="E102" s="34" t="n">
+        <v>35</v>
+      </c>
+      <c r="F102" s="34">
+        <f>D102*E102</f>
+        <v/>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="27" t="inlineStr">
+        <is>
+          <t>Etiquetadora</t>
+        </is>
+      </c>
+      <c r="B103" s="27" t="inlineStr">
+        <is>
+          <t>Etiquetas en blanco</t>
+        </is>
+      </c>
+      <c r="C103" s="28" t="inlineStr">
+        <is>
+          <t>rollo x500</t>
+        </is>
+      </c>
+      <c r="D103" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E103" s="30" t="n">
+        <v>18</v>
+      </c>
+      <c r="F103" s="30">
+        <f>D103*E103</f>
+        <v/>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="31" t="inlineStr">
+        <is>
+          <t>Mesas acero inox</t>
+        </is>
+      </c>
+      <c r="B104" s="31" t="inlineStr">
+        <is>
+          <t>Guantes descartables</t>
+        </is>
+      </c>
+      <c r="C104" s="32" t="inlineStr">
+        <is>
+          <t>caja x100</t>
+        </is>
+      </c>
+      <c r="D104" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="E104" s="34" t="n">
+        <v>18</v>
+      </c>
+      <c r="F104" s="34">
+        <f>D104*E104</f>
+        <v/>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="27" t="inlineStr">
+        <is>
+          <t>Mesas acero inox</t>
+        </is>
+      </c>
+      <c r="B105" s="27" t="inlineStr">
+        <is>
+          <t>Gorros descartables</t>
+        </is>
+      </c>
+      <c r="C105" s="28" t="inlineStr">
+        <is>
+          <t>paquete x100</t>
+        </is>
+      </c>
+      <c r="D105" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E105" s="30" t="n">
+        <v>12</v>
+      </c>
+      <c r="F105" s="30">
+        <f>D105*E105</f>
+        <v/>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="31" t="inlineStr">
+        <is>
+          <t>Mesas acero inox</t>
+        </is>
+      </c>
+      <c r="B106" s="31" t="inlineStr">
+        <is>
+          <t>Mascarillas</t>
+        </is>
+      </c>
+      <c r="C106" s="32" t="inlineStr">
+        <is>
+          <t>paquete x50</t>
+        </is>
+      </c>
+      <c r="D106" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="E106" s="34" t="n">
+        <v>12</v>
+      </c>
+      <c r="F106" s="34">
+        <f>D106*E106</f>
+        <v/>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="27" t="inlineStr">
+        <is>
+          <t>Mesas acero inox</t>
+        </is>
+      </c>
+      <c r="B107" s="27" t="inlineStr">
+        <is>
+          <t>Detergente industrial</t>
+        </is>
+      </c>
+      <c r="C107" s="28" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D107" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E107" s="30" t="n">
+        <v>15</v>
+      </c>
+      <c r="F107" s="30">
+        <f>D107*E107</f>
+        <v/>
+      </c>
+    </row>
+    <row r="108" ht="20" customHeight="1">
+      <c r="A108" s="35" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B108" s="35" t="inlineStr">
+        <is>
+          <t>Industria Alimentaria</t>
+        </is>
+      </c>
+      <c r="C108" s="36" t="n"/>
+      <c r="D108" s="36" t="n"/>
+      <c r="E108" s="36" t="n"/>
+      <c r="F108" s="37">
+        <f>SUM(F97:F107)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="110" ht="22" customHeight="1">
+      <c r="A110" s="25" t="inlineStr">
+        <is>
+          <t>INDUSTRIA DEL VESTIDO</t>
+        </is>
+      </c>
+      <c r="B110" s="25" t="n"/>
+      <c r="C110" s="25" t="n"/>
+      <c r="D110" s="25" t="n"/>
+      <c r="E110" s="25" t="n"/>
+      <c r="F110" s="25" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="26" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+      <c r="B111" s="26" t="inlineStr">
+        <is>
+          <t>Consumible</t>
+        </is>
+      </c>
+      <c r="C111" s="26" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="D111" s="26" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="E111" s="26" t="inlineStr">
+        <is>
+          <t>Precio Unit. (S/.)</t>
+        </is>
+      </c>
+      <c r="F111" s="26" t="inlineStr">
+        <is>
+          <t>Subtotal</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="27" t="inlineStr">
+        <is>
+          <t>Máq. costura industrial</t>
+        </is>
+      </c>
+      <c r="B112" s="27" t="inlineStr">
+        <is>
+          <t>Hilo cono Nro.40 (blanco)</t>
+        </is>
+      </c>
+      <c r="C112" s="28" t="inlineStr">
+        <is>
+          <t>cono</t>
+        </is>
+      </c>
+      <c r="D112" s="29" t="n">
+        <v>2</v>
+      </c>
+      <c r="E112" s="30" t="n">
+        <v>12</v>
+      </c>
+      <c r="F112" s="30">
+        <f>D112*E112</f>
+        <v/>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="31" t="inlineStr">
+        <is>
+          <t>Máq. costura industrial</t>
+        </is>
+      </c>
+      <c r="B113" s="31" t="inlineStr">
+        <is>
+          <t>Hilo cono Nro.40 (colores)</t>
+        </is>
+      </c>
+      <c r="C113" s="32" t="inlineStr">
+        <is>
+          <t>cono</t>
+        </is>
+      </c>
+      <c r="D113" s="33" t="n">
+        <v>3</v>
+      </c>
+      <c r="E113" s="34" t="n">
+        <v>12</v>
+      </c>
+      <c r="F113" s="34">
+        <f>D113*E113</f>
+        <v/>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="27" t="inlineStr">
+        <is>
+          <t>Máq. costura industrial</t>
+        </is>
+      </c>
+      <c r="B114" s="27" t="inlineStr">
+        <is>
+          <t>Agujas industriales 14/90</t>
+        </is>
+      </c>
+      <c r="C114" s="28" t="inlineStr">
+        <is>
+          <t>caja x10</t>
+        </is>
+      </c>
+      <c r="D114" s="29" t="n">
+        <v>2</v>
+      </c>
+      <c r="E114" s="30" t="n">
+        <v>18</v>
+      </c>
+      <c r="F114" s="30">
+        <f>D114*E114</f>
+        <v/>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="31" t="inlineStr">
+        <is>
+          <t>Overlock (remalladora)</t>
+        </is>
+      </c>
+      <c r="B115" s="31" t="inlineStr">
+        <is>
+          <t>Hilos overlock x4 colores</t>
+        </is>
+      </c>
+      <c r="C115" s="32" t="inlineStr">
+        <is>
+          <t>cono</t>
+        </is>
+      </c>
+      <c r="D115" s="33" t="n">
+        <v>8</v>
+      </c>
+      <c r="E115" s="34" t="n">
+        <v>10</v>
+      </c>
+      <c r="F115" s="34">
+        <f>D115*E115</f>
+        <v/>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="27" t="inlineStr">
+        <is>
+          <t>Overlock (remalladora)</t>
+        </is>
+      </c>
+      <c r="B116" s="27" t="inlineStr">
+        <is>
+          <t>Agujas overlock</t>
+        </is>
+      </c>
+      <c r="C116" s="28" t="inlineStr">
+        <is>
+          <t>paquete x10</t>
+        </is>
+      </c>
+      <c r="D116" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E116" s="30" t="n">
+        <v>14</v>
+      </c>
+      <c r="F116" s="30">
+        <f>D116*E116</f>
+        <v/>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="31" t="inlineStr">
+        <is>
+          <t>Recubridora</t>
+        </is>
+      </c>
+      <c r="B117" s="31" t="inlineStr">
+        <is>
+          <t>Hilos recubridora</t>
+        </is>
+      </c>
+      <c r="C117" s="32" t="inlineStr">
+        <is>
+          <t>cono</t>
+        </is>
+      </c>
+      <c r="D117" s="33" t="n">
+        <v>6</v>
+      </c>
+      <c r="E117" s="34" t="n">
+        <v>10</v>
+      </c>
+      <c r="F117" s="34">
+        <f>D117*E117</f>
+        <v/>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="27" t="inlineStr">
+        <is>
+          <t>Recubridora</t>
+        </is>
+      </c>
+      <c r="B118" s="27" t="inlineStr">
+        <is>
+          <t>Agujas recubridora</t>
+        </is>
+      </c>
+      <c r="C118" s="28" t="inlineStr">
+        <is>
+          <t>paquete x5</t>
+        </is>
+      </c>
+      <c r="D118" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E118" s="30" t="n">
+        <v>16</v>
+      </c>
+      <c r="F118" s="30">
+        <f>D118*E118</f>
+        <v/>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="31" t="inlineStr">
+        <is>
+          <t>Cortadora circular</t>
+        </is>
+      </c>
+      <c r="B119" s="31" t="inlineStr">
+        <is>
+          <t>Hoja de corte (reemplazo)</t>
+        </is>
+      </c>
+      <c r="C119" s="32" t="inlineStr">
+        <is>
+          <t>unidad</t>
+        </is>
+      </c>
+      <c r="D119" s="33" t="n">
+        <v>2</v>
+      </c>
+      <c r="E119" s="34" t="n">
+        <v>45</v>
+      </c>
+      <c r="F119" s="34">
+        <f>D119*E119</f>
+        <v/>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="27" t="inlineStr">
+        <is>
+          <t>Plancha industrial</t>
+        </is>
+      </c>
+      <c r="B120" s="27" t="inlineStr">
+        <is>
+          <t>Agua destilada</t>
+        </is>
+      </c>
+      <c r="C120" s="28" t="inlineStr">
+        <is>
+          <t>litro</t>
+        </is>
+      </c>
+      <c r="D120" s="29" t="n">
+        <v>2</v>
+      </c>
+      <c r="E120" s="30" t="n">
+        <v>4</v>
+      </c>
+      <c r="F120" s="30">
+        <f>D120*E120</f>
+        <v/>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="31" t="inlineStr">
+        <is>
+          <t>Material de práctica</t>
+        </is>
+      </c>
+      <c r="B121" s="31" t="inlineStr">
+        <is>
+          <t>Tela popelina básica</t>
+        </is>
+      </c>
+      <c r="C121" s="32" t="inlineStr">
+        <is>
+          <t>metro</t>
+        </is>
+      </c>
+      <c r="D121" s="33" t="n">
+        <v>8</v>
+      </c>
+      <c r="E121" s="34" t="n">
+        <v>8</v>
+      </c>
+      <c r="F121" s="34">
+        <f>D121*E121</f>
+        <v/>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="27" t="inlineStr">
+        <is>
+          <t>Material de práctica</t>
+        </is>
+      </c>
+      <c r="B122" s="27" t="inlineStr">
+        <is>
+          <t>Tela drill 14oz</t>
+        </is>
+      </c>
+      <c r="C122" s="28" t="inlineStr">
+        <is>
+          <t>metro</t>
+        </is>
+      </c>
+      <c r="D122" s="29" t="n">
+        <v>4</v>
+      </c>
+      <c r="E122" s="30" t="n">
+        <v>12</v>
+      </c>
+      <c r="F122" s="30">
+        <f>D122*E122</f>
+        <v/>
+      </c>
+    </row>
+    <row r="123" ht="20" customHeight="1">
+      <c r="A123" s="35" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B123" s="35" t="inlineStr">
+        <is>
+          <t>Industria del Vestido</t>
+        </is>
+      </c>
+      <c r="C123" s="36" t="n"/>
+      <c r="D123" s="36" t="n"/>
+      <c r="E123" s="36" t="n"/>
+      <c r="F123" s="37">
+        <f>SUM(F112:F122)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="125" ht="22" customHeight="1">
+      <c r="A125" s="25" t="inlineStr">
+        <is>
+          <t>MECÁNICA AUTOMOTRIZ</t>
+        </is>
+      </c>
+      <c r="B125" s="25" t="n"/>
+      <c r="C125" s="25" t="n"/>
+      <c r="D125" s="25" t="n"/>
+      <c r="E125" s="25" t="n"/>
+      <c r="F125" s="25" t="n"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="26" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+      <c r="B126" s="26" t="inlineStr">
+        <is>
+          <t>Consumible</t>
+        </is>
+      </c>
+      <c r="C126" s="26" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="D126" s="26" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="E126" s="26" t="inlineStr">
+        <is>
+          <t>Precio Unit. (S/.)</t>
+        </is>
+      </c>
+      <c r="F126" s="26" t="inlineStr">
+        <is>
+          <t>Subtotal</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="27" t="inlineStr">
+        <is>
+          <t>Elevador hidráulico</t>
+        </is>
+      </c>
+      <c r="B127" s="27" t="inlineStr">
+        <is>
+          <t>Aceite hidráulico ISO 46</t>
+        </is>
+      </c>
+      <c r="C127" s="28" t="inlineStr">
+        <is>
+          <t>litro</t>
+        </is>
+      </c>
+      <c r="D127" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E127" s="30" t="n">
+        <v>22</v>
+      </c>
+      <c r="F127" s="30">
+        <f>D127*E127</f>
+        <v/>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="31" t="inlineStr">
+        <is>
+          <t>Desmontadora neumáticos</t>
+        </is>
+      </c>
+      <c r="B128" s="31" t="inlineStr">
+        <is>
+          <t>Lubricante de montaje</t>
+        </is>
+      </c>
+      <c r="C128" s="32" t="inlineStr">
+        <is>
+          <t>litro</t>
+        </is>
+      </c>
+      <c r="D128" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="E128" s="34" t="n">
+        <v>18</v>
+      </c>
+      <c r="F128" s="34">
+        <f>D128*E128</f>
+        <v/>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="27" t="inlineStr">
+        <is>
+          <t>Balanceadora</t>
+        </is>
+      </c>
+      <c r="B129" s="27" t="inlineStr">
+        <is>
+          <t>Pesas adhesivas balanceo</t>
+        </is>
+      </c>
+      <c r="C129" s="28" t="inlineStr">
+        <is>
+          <t>caja 100u</t>
+        </is>
+      </c>
+      <c r="D129" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E129" s="30" t="n">
+        <v>48</v>
+      </c>
+      <c r="F129" s="30">
+        <f>D129*E129</f>
+        <v/>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="31" t="inlineStr">
+        <is>
+          <t>Compresor de aire</t>
+        </is>
+      </c>
+      <c r="B130" s="31" t="inlineStr">
+        <is>
+          <t>Aceite para compresor</t>
+        </is>
+      </c>
+      <c r="C130" s="32" t="inlineStr">
+        <is>
+          <t>litro</t>
+        </is>
+      </c>
+      <c r="D130" s="33" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E130" s="34" t="n">
+        <v>25</v>
+      </c>
+      <c r="F130" s="34">
+        <f>D130*E130</f>
+        <v/>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="27" t="inlineStr">
+        <is>
+          <t>Práctica cambio aceite</t>
+        </is>
+      </c>
+      <c r="B131" s="27" t="inlineStr">
+        <is>
+          <t>Aceite motor 15W40</t>
+        </is>
+      </c>
+      <c r="C131" s="28" t="inlineStr">
+        <is>
+          <t>litro</t>
+        </is>
+      </c>
+      <c r="D131" s="29" t="n">
+        <v>4</v>
+      </c>
+      <c r="E131" s="30" t="n">
+        <v>14</v>
+      </c>
+      <c r="F131" s="30">
+        <f>D131*E131</f>
+        <v/>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="31" t="inlineStr">
+        <is>
+          <t>Práctica cambio aceite</t>
+        </is>
+      </c>
+      <c r="B132" s="31" t="inlineStr">
+        <is>
+          <t>Filtro de aceite</t>
+        </is>
+      </c>
+      <c r="C132" s="32" t="inlineStr">
+        <is>
+          <t>unidad</t>
+        </is>
+      </c>
+      <c r="D132" s="33" t="n">
+        <v>2</v>
+      </c>
+      <c r="E132" s="34" t="n">
+        <v>28</v>
+      </c>
+      <c r="F132" s="34">
+        <f>D132*E132</f>
+        <v/>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="27" t="inlineStr">
+        <is>
+          <t>Práctica cambio aceite</t>
+        </is>
+      </c>
+      <c r="B133" s="27" t="inlineStr">
+        <is>
+          <t>Trapo industrial</t>
+        </is>
+      </c>
+      <c r="C133" s="28" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D133" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E133" s="30" t="n">
+        <v>12</v>
+      </c>
+      <c r="F133" s="30">
+        <f>D133*E133</f>
+        <v/>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="31" t="inlineStr">
+        <is>
+          <t>Práctica de frenos</t>
+        </is>
+      </c>
+      <c r="B134" s="31" t="inlineStr">
+        <is>
+          <t>Pastillas de freno (par)</t>
+        </is>
+      </c>
+      <c r="C134" s="32" t="inlineStr">
+        <is>
+          <t>par</t>
+        </is>
+      </c>
+      <c r="D134" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="E134" s="34" t="n">
+        <v>48</v>
+      </c>
+      <c r="F134" s="34">
+        <f>D134*E134</f>
+        <v/>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="27" t="inlineStr">
+        <is>
+          <t>Práctica de frenos</t>
+        </is>
+      </c>
+      <c r="B135" s="27" t="inlineStr">
+        <is>
+          <t>Líquido de frenos DOT4</t>
+        </is>
+      </c>
+      <c r="C135" s="28" t="inlineStr">
+        <is>
+          <t>frasco 500ml</t>
+        </is>
+      </c>
+      <c r="D135" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E135" s="30" t="n">
+        <v>22</v>
+      </c>
+      <c r="F135" s="30">
+        <f>D135*E135</f>
+        <v/>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="31" t="inlineStr">
+        <is>
+          <t>Práctica de frenos</t>
+        </is>
+      </c>
+      <c r="B136" s="31" t="inlineStr">
+        <is>
+          <t>Limpiador de frenos</t>
+        </is>
+      </c>
+      <c r="C136" s="32" t="inlineStr">
+        <is>
+          <t>spray 400ml</t>
+        </is>
+      </c>
+      <c r="D136" s="33" t="n">
+        <v>2</v>
+      </c>
+      <c r="E136" s="34" t="n">
+        <v>18</v>
+      </c>
+      <c r="F136" s="34">
+        <f>D136*E136</f>
+        <v/>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="27" t="inlineStr">
+        <is>
+          <t>Escáner diagnóstico</t>
+        </is>
+      </c>
+      <c r="B137" s="27" t="inlineStr">
+        <is>
+          <t>Cable OBD2 repuesto</t>
+        </is>
+      </c>
+      <c r="C137" s="28" t="inlineStr">
+        <is>
+          <t>unidad</t>
+        </is>
+      </c>
+      <c r="D137" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E137" s="30" t="n">
+        <v>35</v>
+      </c>
+      <c r="F137" s="30">
+        <f>D137*E137</f>
+        <v/>
+      </c>
+    </row>
+    <row r="138" ht="20" customHeight="1">
+      <c r="A138" s="35" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B138" s="35" t="inlineStr">
+        <is>
+          <t>Mecánica Automotriz</t>
+        </is>
+      </c>
+      <c r="C138" s="36" t="n"/>
+      <c r="D138" s="36" t="n"/>
+      <c r="E138" s="36" t="n"/>
+      <c r="F138" s="37">
+        <f>SUM(F127:F137)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="141" ht="22" customHeight="1">
+      <c r="A141" s="38" t="inlineStr">
+        <is>
+          <t>Especialidad</t>
+        </is>
+      </c>
+      <c r="B141" s="38" t="inlineStr">
+        <is>
+          <t>Total Consumibles (S/.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="27" t="inlineStr">
+        <is>
+          <t>Cocina y Repostería</t>
+        </is>
+      </c>
+      <c r="B142" s="39">
+        <f>F17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="31" t="inlineStr">
+        <is>
+          <t>Computación e Informática</t>
+        </is>
+      </c>
+      <c r="B143" s="40">
+        <f>F29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="27" t="inlineStr">
+        <is>
+          <t>Construcciones Metálicas</t>
+        </is>
+      </c>
+      <c r="B144" s="39">
+        <f>F45</f>
+        <v/>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="31" t="inlineStr">
+        <is>
+          <t>Ebanistería</t>
+        </is>
+      </c>
+      <c r="B145" s="40">
+        <f>F62</f>
+        <v/>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="27" t="inlineStr">
+        <is>
+          <t>Electricidad</t>
+        </is>
+      </c>
+      <c r="B146" s="39">
+        <f>F77</f>
+        <v/>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="31" t="inlineStr">
+        <is>
+          <t>Electrónica</t>
+        </is>
+      </c>
+      <c r="B147" s="40">
+        <f>F93</f>
+        <v/>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="27" t="inlineStr">
+        <is>
+          <t>Industria Alimentaria</t>
+        </is>
+      </c>
+      <c r="B148" s="39">
+        <f>F108</f>
+        <v/>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="31" t="inlineStr">
+        <is>
+          <t>Industria del Vestido</t>
+        </is>
+      </c>
+      <c r="B149" s="40">
+        <f>F123</f>
+        <v/>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="27" t="inlineStr">
+        <is>
+          <t>Mecánica Automotriz</t>
+        </is>
+      </c>
+      <c r="B150" s="39">
+        <f>F138</f>
+        <v/>
+      </c>
+    </row>
+    <row r="151" ht="22" customHeight="1">
+      <c r="A151" s="41" t="inlineStr">
+        <is>
+          <t>GRAN TOTAL CONSUMIBLES</t>
+        </is>
+      </c>
+      <c r="B151" s="42">
+        <f>SUM(B142:B150)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4368,7 +7966,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4589,7 +8187,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>